<commit_message>
Add CR materiality threshold; make in-year savings primacy explicit
- Guiding principles: change requests required (and baseline restated)
  only for changes with $500K+ in-year savings impact in any year;
  sub-threshold items handled via commentary with baseline unchanged;
  no splitting to dodge the threshold. Added to open questions.
- Guiding principles & strategy assessment: in-year savings vs. the
  2025-2029 committed targets is the accountability metric; exit
  run-rate is diagnostic only and never offsets an in-year miss.
- Workbook Guiding Principles tab updated to match; regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N9N7wxtcxHnjJY1MmKUtRB
</commit_message>
<xml_diff>
--- a/india-labor-arbitrage/India_Labor_Arbitrage_Tracker.xlsx
+++ b/india-labor-arbitrage/India_Labor_Arbitrage_Tracker.xlsx
@@ -20432,7 +20432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -20451,7 +20451,7 @@
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="31" t="inlineStr">
         <is>
-          <t>1. The baseline is the committed monthly target loaded to your forecast. Variances are vs. that baseline — never vs. prior year or re-forecast. Baseline moves only via approved change request.</t>
+          <t>1. The baseline is the committed monthly target loaded to your forecast. Variances are vs. that baseline — never vs. prior year or re-forecast. Baseline moves only via approved change request, required for changes with in-year savings impact of $500K+ in any year (proposed threshold); smaller items are handled via commentary and do NOT restate the baseline.</t>
         </is>
       </c>
     </row>
@@ -20486,26 +20486,33 @@
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="31" t="inlineStr">
         <is>
-          <t>6. Recognize savings in the month the run-rate reduction first hits the GL — not at contract signature or vendor notification. Partial months pro rata.</t>
+          <t>5a. IN-YEAR IS THE COMMITMENT: the enterprise committed in-year savings targets by year for 2025-2029, allocated by sub-organization. Exit run-rate is a diagnostic only — being 'on track on run-rate' never offsets or excuses an in-year miss. Run-rate belongs in recovery-plan commentary, not the scorecard.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="31" t="inlineStr">
         <is>
-          <t>7. No leakage: a reduction is not real if equivalent spend reappears in another cost center, vendor, or expense line. You attest to this monthly.</t>
+          <t>6. Recognize savings in the month the run-rate reduction first hits the GL — not at contract signature or vendor notification. Partial months pro rata.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="31" t="inlineStr">
         <is>
-          <t>8. Attestation &amp; evidence: the org finance partner attests each submission and can identify the cost center and expense line for material reductions on request. Quarterly sample testing and true-up apply.</t>
+          <t>7. No leakage: a reduction is not real if equivalent spend reappears in another cost center, vendor, or expense line. You attest to this monthly.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>8. Attestation &amp; evidence: the org finance partner attests each submission and can identify the cost center and expense line for material reductions on request. Quarterly sample testing and true-up apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>9. When in doubt, ask central program finance BEFORE reporting the number. Interpretation rulings are appended to the full Guiding Principles document.</t>
         </is>

</xml_diff>